<commit_message>
GFORMS-4673 Update resource file as per MCI-5 request (#2742)
(cherry picked from commit 0acf999749825d42947341b61240793acee31161)
</commit_message>
<xml_diff>
--- a/conf/resources/goods-and-services-after-deregistered-schedule-cy.xlsx
+++ b/conf/resources/goods-and-services-after-deregistered-schedule-cy.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emmamorton/Documents/Projects/gForms/VAT forms/Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hmrc-my.sharepoint.com/personal/katrin_lloyd_hmrc_gov_uk/Documents/Desktop/!! VERSIONS TERFYNOL !!/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F1F5666-B6BF-1449-8451-7770F7F3E02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{5E3822F8-748C-4837-87E1-DE65787270A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B43153F-E1A7-414C-BEA5-AF6A36574811}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="VAT Reclaim Form" sheetId="1" r:id="rId1"/>
+    <sheet name="Cover" sheetId="2" r:id="rId1"/>
+    <sheet name="Ffurflen Adhawlio TAW" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,88 +34,168 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>Disgrifiad o’r Nwyddau</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+  <si>
+    <t>Ffurflen Adhawlio TAW</t>
+  </si>
+  <si>
+    <t>Mae’r daflen waith hon yn cynnwys nodiadau i’ch helpu i lenwi’r tabl ar y daflen waith ‘Manylion yr hawliad’.</t>
+  </si>
+  <si>
+    <t>Cyhoeddwyd gan CThEF ar 9 Gorffennaf 2026.</t>
+  </si>
+  <si>
+    <t>Enw’r golofn ar y daflen waith ‘Manylion yr hawliad’</t>
+  </si>
+  <si>
+    <t>Nodiadau ac enghreifftiau</t>
+  </si>
+  <si>
+    <t>Cell y golofn ar y daflen waith ‘Manylion yr hawliad’</t>
+  </si>
+  <si>
+    <t>Enw’r person neu’r busnes a ddarparodd y nwyddau neu’r gwasanaethau (fel y mae’n ymddangos ar yr anfoneb)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nodwch enw’r darparwr fel y mae’n ymddangos ar yr anfoneb.
+</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>Rhif yr anfoneb/ Rhif y Nodyn Credyd</t>
+  </si>
+  <si>
+    <t>Bydd hyn i’w weld ar yr anfoneb neu’r nodyn credyd.</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>Y math o ddogfen gwerthiannau</t>
+  </si>
+  <si>
+    <t>Anfoneb neu Nodyn Credyd</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>Y dyddiad y cafodd yr anfoneb neu’r nodyn credyd ei anfon</t>
+  </si>
+  <si>
+    <t>Bydd hyn i’w weld ar yr anfoneb. Er enghraifft, 19 3 2022.</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>Amser cyflenwi (y pwynt treth)</t>
+  </si>
+  <si>
+    <t>Yr amser cyflenwi yw’r dyddiad y daw anfoneb yn drethadwy. Yn y rhan fwyaf o achosion, dyma’r dyddiad yr anfonwyd yr anfoneb. Fodd bynnag, nid yw hyn bob amser yn wir. I wirio eich pwynt treth, ewch i adran 14 o Hysbysiad TAW 700</t>
+  </si>
+  <si>
+    <t>E1</t>
+  </si>
+  <si>
+    <t>Swm y TAW rydych chi’n adhawlio ar yr anfoneb, neu swm y TAW sydd heb ei dalu ar y nodyn credyd (nodwch y swm mewn GBP)</t>
+  </si>
+  <si>
+    <t>Rhowch swm y TAW i’w hawlio yn seiliedig ar yr anfoneb ategol neu’r nodyn credyd ategol. Dylid nodi symiau nodau credyd fel gwerthoedd negyddol</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>Disgrifiad o’r nwyddau neu’r gwasanaethau</t>
+  </si>
+  <si>
+    <t>Disgrifiwch y nwyddau neu’r gwasanaethau rydych chi am adhawlio TAW ar eu cyfer.
+Rhowch ddisgrifiad byr, fel ‘Cadeiriau ar gyfer ystafell fwyta’ neu ‘Ford Focus’.</t>
+  </si>
+  <si>
+    <t>G1</t>
   </si>
   <si>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
+      </rPr>
+      <t>Enw’r person neu’r busnes a ddarparodd y nwyddau neu’r gwasanaethau</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (fel y mae’n ymddangos ar yr anfoneb neu’r nodyn credyd)</t>
+    </r>
+  </si>
+  <si>
+    <t>Rhif yr Anfoneb neu Rif y Nodyn Credyd</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Y math o ddogfen gwerthiannau </t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
       <t>(anfoneb, neu nodyn credyd)</t>
     </r>
   </si>
   <si>
+    <t>Amser Cyflenwi</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Enw’r person neu’r busnes a ddarperir y nwyddau neu’r gwasanaethau </t>
+      <t>Swm y TAW rydych chi’n adhawlio ar yr anfoneb, neu swm y TAW sydd heb ei dalu ar y nodyn credyd</t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (fel y mae’n ymddangos ar yr anfoneb neu’r nodyn credyd)</t>
-    </r>
-  </si>
-  <si>
-    <t>Y dyddiad y cafodd yr anfoneb neu’r nodyn credyd ei anfon</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Swm y TAW rydych chi’n adhawlio ar yr anfoneb, neu’r swm y TAW sy’n parhau i fod heb ei dalu ar y nodyn credyd</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> (nodwch y swm mewn GBP)</t>
     </r>
+  </si>
+  <si>
+    <t>Disgrifiad o’r Nwyddau neu’r Gwasanaethau</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,51 +205,82 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0B0C0C"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="16"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <sz val="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -176,26 +288,208 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{1D8DE468-AF24-4049-95AE-C197458D9C55}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -206,6 +500,22 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63C6995B-2C67-49BE-A101-FBE7BEE47DEC}" name="NotesTable" displayName="NotesTable" ref="A3:C10" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A3:C10" xr:uid="{02D23C97-5724-4035-ABFD-053F6EC6ADA9}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{EC64CF77-8644-4AA2-AED4-62096FDD7E98}" name="Enw’r golofn ar y daflen waith ‘Manylion yr hawliad’" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{68AA6B9B-58C0-435F-BAAD-B1ED5C3805B0}" name="Nodiadau ac enghreifftiau" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{53FEC9E7-954A-4712-B03C-DFC9280FC815}" name="Cell y golofn ar y daflen waith ‘Manylion yr hawliad’" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -492,63 +802,211 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE20D863-C1FE-4BA4-B947-BF0214F0F4AF}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="38.33203125" customWidth="1"/>
-    <col min="2" max="2" width="20.5" customWidth="1"/>
-    <col min="3" max="3" width="31.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
-    <col min="5" max="5" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="69" style="1" customWidth="1"/>
+    <col min="2" max="2" width="73.42578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" ht="80" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="43.5" customHeight="1">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" ht="42" customHeight="1">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C2" s="11"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" ht="47.25">
+      <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="B3" s="10" t="s">
         <v>4</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" ht="50.1" customHeight="1">
+      <c r="A4" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" ht="41.1" customHeight="1">
+      <c r="A5" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" ht="41.1" customHeight="1">
+      <c r="A6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="71.45" customHeight="1">
+      <c r="A7" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="64.5" customHeight="1">
+      <c r="A8" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="65.099999999999994" customHeight="1">
+      <c r="A9" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="65.099999999999994" customHeight="1">
+      <c r="A10" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1">
+      <c r="A11" s="4"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1">
+      <c r="A12" s="4"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="28.28515625" customWidth="1"/>
+    <col min="7" max="7" width="49" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="26" customFormat="1" ht="93.75">
+      <c r="A1" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 OFFICIAL</oddFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;&amp;"Calibri"&amp;10&amp;K000000 SWYDDOGOL</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="78648aa0-189c-4913-b480-8f083842eefa">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="252b28bd-d93f-4b99-825e-07b76ab2fd6b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D23464B46C9A6C438A9A63FA525492B5" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="816d63d098657adee5e1780dd4373ff3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="78648aa0-189c-4913-b480-8f083842eefa" xmlns:ns3="252b28bd-d93f-4b99-825e-07b76ab2fd6b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cc6b77c161da750edc5730dfe65423ec" ns2:_="" ns3:_="">
     <xsd:import namespace="78648aa0-189c-4913-b480-8f083842eefa"/>
@@ -797,26 +1255,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7BD096F-CBD5-47C0-BAA0-60D61AFDFDD3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A280DCCB-AF13-4408-B828-DBA969B42C4A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="78648aa0-189c-4913-b480-8f083842eefa"/>
-    <ds:schemaRef ds:uri="252b28bd-d93f-4b99-825e-07b76ab2fd6b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="78648aa0-189c-4913-b480-8f083842eefa">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="252b28bd-d93f-4b99-825e-07b76ab2fd6b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0ED3C42-CCAD-47EF-8277-49E5144C7C18}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -833,4 +1292,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7BD096F-CBD5-47C0-BAA0-60D61AFDFDD3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A280DCCB-AF13-4408-B828-DBA969B42C4A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="78648aa0-189c-4913-b480-8f083842eefa"/>
+    <ds:schemaRef ds:uri="252b28bd-d93f-4b99-825e-07b76ab2fd6b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f9af038e-07b4-4369-a678-c835687cb272}" enabled="1" method="Standard" siteId="{ac52f73c-fd1a-4a9a-8e7a-4a248f3139e1}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>